<commit_message>
Add web-sourced figures: remittances ~8% GDP, female LFP 19%, ECI rank #78 (orange=verify)
</commit_message>
<xml_diff>
--- a/THE_MOROCCO_EQUATION_DATABASE.xlsx
+++ b/THE_MOROCCO_EQUATION_DATABASE.xlsx
@@ -56,7 +56,7 @@
     </font>
     <font/>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +88,11 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -115,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -178,6 +183,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -517,6 +525,71 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>web-search</author>
+  </authors>
+  <commentList>
+    <comment ref="I4" authorId="0" shapeId="0">
+      <text>
+        <t>[C] 2024 remittances ~MAD 116.28bn. Source: Office des Changes via press, 2025. VERIFY.</t>
+      </text>
+    </comment>
+    <comment ref="J4" authorId="0" shapeId="0">
+      <text>
+        <t>[C] 2025 remittances ~MAD 122bn (+2.6% YoY). Source: Office des Changes, reported via Atalayar/AceMoneyTransfer, 2026. VERIFY exact OC figure.</t>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0">
+      <text>
+        <t>[G] 2020 remittances 6.46% of GDP (World Bank/TradingEconomics).</t>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="0" shapeId="0">
+      <text>
+        <t>[G] 2024 remittances ~8% of GDP (World Bank; Statista 7.79%). VERIFY exact %.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>web-search</author>
+  </authors>
+  <commentList>
+    <comment ref="G4" authorId="0" shapeId="0">
+      <text>
+        <t>[A/G] 2023 female LFP 19% (HCP, via Policy Center 2024; World Bank confirms). 15+ definition.</t>
+      </text>
+    </comment>
+    <comment ref="H4" authorId="0" shapeId="0">
+      <text>
+        <t>[A] Q1-2026 female LFP 17.5% (HCP, via Morocco World News May-2026). NOTE: declining. 2024 was 19.1%.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>web-search</author>
+  </authors>
+  <commentList>
+    <comment ref="H3" authorId="0" shapeId="0">
+      <text>
+        <t>OEC (oec.world) ranks Morocco #78 most complex economy (latest). NOTE: this is OEC methodology, NOT Harvard Atlas. Manuscript cites Harvard Atlas - pull the Harvard number from atlas.hks.harvard.edu and VERIFY it agrees. Our World in Data also has the series.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1056,8 +1129,12 @@
       <c r="D4" s="14" t="n"/>
       <c r="E4" s="14" t="n"/>
       <c r="F4" s="14" t="n"/>
-      <c r="G4" s="14" t="n"/>
-      <c r="H4" s="14" t="n"/>
+      <c r="G4" s="26" t="n">
+        <v>19</v>
+      </c>
+      <c r="H4" s="26" t="n">
+        <v>17.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -1100,7 +1177,7 @@
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Female LFP replaces [X] in TEXT-16. Water 1960s≈2500, threshold=1000. [A][G][L].</t>
+          <t>FEMALE LFP FOUND (orange=verify): 19% (2023) -&gt; 19.1% (2024) -&gt; 17.5% (Q1-2026, HCP). DECLINING. Use ~19% in TEXT-16 but note the decline. Caution: World Bank 'modeled, 15-64' shows ~21% (different definition) - use HCP 15+ for consistency.</t>
         </is>
       </c>
     </row>
@@ -1111,6 +1188,7 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1198,7 +1276,9 @@
       <c r="E3" s="14" t="n"/>
       <c r="F3" s="14" t="n"/>
       <c r="G3" s="14" t="n"/>
-      <c r="H3" s="14" t="n"/>
+      <c r="H3" s="26" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -1235,6 +1315,13 @@
       <c r="F5" s="14" t="n"/>
       <c r="G5" s="14" t="n"/>
       <c r="H5" s="14" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ECI: OEC ranks Morocco #78 (latest). MUST pull Harvard Atlas figure separately (different methodology) AND verify the multi-year DIRECTION before writing 'moved materially up'. [H] atlas.hks.harvard.edu ; cross-check ourworldindata.org/grapher/economic-complexity-rankings.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -1250,6 +1337,7 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -4918,8 +5006,12 @@
       <c r="F4" s="14" t="n"/>
       <c r="G4" s="14" t="n"/>
       <c r="H4" s="14" t="n"/>
-      <c r="I4" s="14" t="n"/>
-      <c r="J4" s="14" t="n"/>
+      <c r="I4" s="26" t="n">
+        <v>116.28</v>
+      </c>
+      <c r="J4" s="26" t="n">
+        <v>122</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -4934,11 +5026,15 @@
       </c>
       <c r="C5" s="14" t="n"/>
       <c r="D5" s="14" t="n"/>
-      <c r="E5" s="14" t="n"/>
+      <c r="E5" s="26" t="n">
+        <v>6.46</v>
+      </c>
       <c r="F5" s="14" t="n"/>
       <c r="G5" s="14" t="n"/>
       <c r="H5" s="14" t="n"/>
-      <c r="I5" s="14" t="n"/>
+      <c r="I5" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="J5" s="14" t="n"/>
     </row>
     <row r="6">
@@ -5010,7 +5106,7 @@
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>Feeds TEXT-7 + FIG-3b. Confirm remittances % to replace [X]. [C] Office des Changes; [E] BAM; [F] IMF.</t>
+          <t>REMITTANCES FOUND (orange=verify): 2024 ~8% GDP / ~MAD116bn; 2025 ~MAD122bn (+2.6%). Replace [X] in TEXT-7 with ~8%. [C] Office des Changes; [G] World Bank.</t>
         </is>
       </c>
     </row>
@@ -5021,6 +5117,7 @@
     <mergeCell ref="A10:J11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>